<commit_message>
Refactor ATOM downloader; update data files
Refactor KOTAK_DB notebook Selenium downloader: switch to Path-based BASE_DIR, update download paths to kotak-salesian-school-dbms, add webdriver_manager usage, improved wait/download logic, add helpers (set_dates, has_no_records), remove old atom_report.xlsx before run, use Path.unlink, increase timeouts and print clearer messages, and bump nbformat python version. Also add a new transaction Excel (source_data/Transaction_file20260207-154636.xlsx), replace atom_report.xlsx, and apply corrections to many rows in merged_fee_collection.csv (fee/paid/due fixes).
</commit_message>
<xml_diff>
--- a/source_data/atom_report.xlsx
+++ b/source_data/atom_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BV312"/>
+  <dimension ref="A1:BV317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62022,6 +62022,942 @@
         </is>
       </c>
     </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>753702</v>
+      </c>
+      <c r="C313" t="n">
+        <v>1234</v>
+      </c>
+      <c r="D313" t="n">
+        <v>11000348990079</v>
+      </c>
+      <c r="E313" t="n">
+        <v>1770372650</v>
+      </c>
+      <c r="F313" t="n">
+        <v>8050</v>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>06-Feb-2026 15:42:50</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="N313" t="n">
+        <v>696631043153</v>
+      </c>
+      <c r="O313" t="inlineStr"/>
+      <c r="P313" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R313" t="inlineStr">
+        <is>
+          <t>07-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="S313" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T313" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U313" t="inlineStr"/>
+      <c r="V313" t="inlineStr"/>
+      <c r="W313" t="inlineStr"/>
+      <c r="X313" t="inlineStr"/>
+      <c r="Y313" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z313" t="n">
+        <v>9542502425</v>
+      </c>
+      <c r="AA313" t="inlineStr"/>
+      <c r="AB313" t="inlineStr"/>
+      <c r="AC313" t="inlineStr"/>
+      <c r="AD313" t="inlineStr"/>
+      <c r="AE313" t="inlineStr"/>
+      <c r="AF313" t="inlineStr"/>
+      <c r="AG313" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH313" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AI313" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ313" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK313" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AL313" t="n">
+        <v>8050</v>
+      </c>
+      <c r="AM313" t="inlineStr">
+        <is>
+          <t>07-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="AN313" t="inlineStr"/>
+      <c r="AO313" t="inlineStr"/>
+      <c r="AP313" t="inlineStr"/>
+      <c r="AQ313" t="inlineStr"/>
+      <c r="AR313" t="inlineStr"/>
+      <c r="AS313" t="inlineStr"/>
+      <c r="AT313" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU313" t="inlineStr"/>
+      <c r="AV313" t="inlineStr"/>
+      <c r="AW313" t="inlineStr"/>
+      <c r="AX313" t="inlineStr"/>
+      <c r="AY313" t="inlineStr"/>
+      <c r="AZ313" t="inlineStr"/>
+      <c r="BA313" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB313" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC313" t="inlineStr"/>
+      <c r="BD313" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE313" t="n">
+        <v>18422</v>
+      </c>
+      <c r="BF313" t="inlineStr">
+        <is>
+          <t>267145</t>
+        </is>
+      </c>
+      <c r="BG313" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="BH313" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="BI313" t="n">
+        <v>16400</v>
+      </c>
+      <c r="BJ313" t="inlineStr"/>
+      <c r="BK313" t="inlineStr"/>
+      <c r="BL313" t="inlineStr"/>
+      <c r="BM313" t="inlineStr"/>
+      <c r="BN313" t="inlineStr"/>
+      <c r="BO313" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+      <c r="BP313" t="inlineStr"/>
+      <c r="BQ313" t="inlineStr"/>
+      <c r="BR313" t="inlineStr"/>
+      <c r="BS313" t="inlineStr"/>
+      <c r="BT313" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU313" t="inlineStr"/>
+      <c r="BV313" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>753702</v>
+      </c>
+      <c r="C314" t="n">
+        <v>1234</v>
+      </c>
+      <c r="D314" t="n">
+        <v>11000349086368</v>
+      </c>
+      <c r="E314" t="n">
+        <v>1770445075</v>
+      </c>
+      <c r="F314" t="n">
+        <v>8350</v>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>07-Feb-2026 11:49:02</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N314" t="n">
+        <v>109145651654</v>
+      </c>
+      <c r="O314" t="inlineStr"/>
+      <c r="P314" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="Q314" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R314" t="inlineStr"/>
+      <c r="S314" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T314" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U314" t="inlineStr"/>
+      <c r="V314" t="inlineStr"/>
+      <c r="W314" t="inlineStr"/>
+      <c r="X314" t="inlineStr"/>
+      <c r="Y314" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z314" t="n">
+        <v>9505890135</v>
+      </c>
+      <c r="AA314" t="inlineStr"/>
+      <c r="AB314" t="inlineStr"/>
+      <c r="AC314" t="inlineStr"/>
+      <c r="AD314" t="inlineStr"/>
+      <c r="AE314" t="inlineStr"/>
+      <c r="AF314" t="inlineStr"/>
+      <c r="AG314" t="inlineStr"/>
+      <c r="AH314" t="inlineStr"/>
+      <c r="AI314" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ314" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK314" t="inlineStr"/>
+      <c r="AL314" t="inlineStr"/>
+      <c r="AM314" t="inlineStr"/>
+      <c r="AN314" t="inlineStr"/>
+      <c r="AO314" t="inlineStr"/>
+      <c r="AP314" t="inlineStr"/>
+      <c r="AQ314" t="inlineStr"/>
+      <c r="AR314" t="inlineStr"/>
+      <c r="AS314" t="inlineStr"/>
+      <c r="AT314" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU314" t="inlineStr"/>
+      <c r="AV314" t="inlineStr"/>
+      <c r="AW314" t="inlineStr"/>
+      <c r="AX314" t="inlineStr"/>
+      <c r="AY314" t="inlineStr"/>
+      <c r="AZ314" t="inlineStr"/>
+      <c r="BA314" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB314" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC314" t="inlineStr"/>
+      <c r="BD314" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE314" t="n">
+        <v>18805</v>
+      </c>
+      <c r="BF314" t="inlineStr">
+        <is>
+          <t>267429</t>
+        </is>
+      </c>
+      <c r="BG314" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="BH314" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI314" t="n">
+        <v>15762</v>
+      </c>
+      <c r="BJ314" t="inlineStr"/>
+      <c r="BK314" t="inlineStr"/>
+      <c r="BL314" t="inlineStr"/>
+      <c r="BM314" t="inlineStr"/>
+      <c r="BN314" t="inlineStr"/>
+      <c r="BO314" t="inlineStr"/>
+      <c r="BP314" t="inlineStr"/>
+      <c r="BQ314" t="inlineStr"/>
+      <c r="BR314" t="inlineStr"/>
+      <c r="BS314" t="inlineStr"/>
+      <c r="BT314" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU314" t="inlineStr"/>
+      <c r="BV314" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>753702</v>
+      </c>
+      <c r="C315" t="n">
+        <v>1234</v>
+      </c>
+      <c r="D315" t="n">
+        <v>11000349179233</v>
+      </c>
+      <c r="E315" t="n">
+        <v>1770528801</v>
+      </c>
+      <c r="F315" t="n">
+        <v>8350</v>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>08-Feb-2026 11:04:35</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDFC Bank </t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N315" t="inlineStr"/>
+      <c r="O315" t="inlineStr"/>
+      <c r="P315" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="Q315" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R315" t="inlineStr"/>
+      <c r="S315" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T315" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="U315" t="inlineStr"/>
+      <c r="V315" t="inlineStr"/>
+      <c r="W315" t="inlineStr"/>
+      <c r="X315" t="inlineStr"/>
+      <c r="Y315" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z315" t="n">
+        <v>6305761566</v>
+      </c>
+      <c r="AA315" t="inlineStr"/>
+      <c r="AB315" t="inlineStr"/>
+      <c r="AC315" t="inlineStr"/>
+      <c r="AD315" t="inlineStr"/>
+      <c r="AE315" t="inlineStr"/>
+      <c r="AF315" t="inlineStr"/>
+      <c r="AG315" t="inlineStr"/>
+      <c r="AH315" t="inlineStr"/>
+      <c r="AI315" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ315" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK315" t="inlineStr"/>
+      <c r="AL315" t="inlineStr"/>
+      <c r="AM315" t="inlineStr"/>
+      <c r="AN315" t="inlineStr"/>
+      <c r="AO315" t="inlineStr"/>
+      <c r="AP315" t="inlineStr"/>
+      <c r="AQ315" t="inlineStr"/>
+      <c r="AR315" t="inlineStr"/>
+      <c r="AS315" t="inlineStr"/>
+      <c r="AT315" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS FAILED</t>
+        </is>
+      </c>
+      <c r="AU315" t="inlineStr"/>
+      <c r="AV315" t="inlineStr"/>
+      <c r="AW315" t="inlineStr"/>
+      <c r="AX315" t="inlineStr"/>
+      <c r="AY315" t="inlineStr"/>
+      <c r="AZ315" t="inlineStr"/>
+      <c r="BA315" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="BB315" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC315" t="inlineStr"/>
+      <c r="BD315" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE315" t="n">
+        <v>19972</v>
+      </c>
+      <c r="BF315" t="inlineStr">
+        <is>
+          <t>265869</t>
+        </is>
+      </c>
+      <c r="BG315" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="BH315" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI315" t="n">
+        <v>17260</v>
+      </c>
+      <c r="BJ315" t="inlineStr"/>
+      <c r="BK315" t="inlineStr"/>
+      <c r="BL315" t="inlineStr"/>
+      <c r="BM315" t="inlineStr"/>
+      <c r="BN315" t="inlineStr"/>
+      <c r="BO315" t="inlineStr"/>
+      <c r="BP315" t="inlineStr"/>
+      <c r="BQ315" t="inlineStr"/>
+      <c r="BR315" t="inlineStr"/>
+      <c r="BS315" t="inlineStr"/>
+      <c r="BT315" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU315" t="inlineStr"/>
+      <c r="BV315" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>753702</v>
+      </c>
+      <c r="C316" t="n">
+        <v>1234</v>
+      </c>
+      <c r="D316" t="n">
+        <v>11000349188445</v>
+      </c>
+      <c r="E316" t="n">
+        <v>1770534277</v>
+      </c>
+      <c r="F316" t="n">
+        <v>8350</v>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>08-Feb-2026 12:35:23</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N316" t="n">
+        <v>773499900668</v>
+      </c>
+      <c r="O316" t="inlineStr"/>
+      <c r="P316" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="Q316" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R316" t="inlineStr"/>
+      <c r="S316" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T316" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U316" t="inlineStr"/>
+      <c r="V316" t="inlineStr"/>
+      <c r="W316" t="inlineStr"/>
+      <c r="X316" t="inlineStr"/>
+      <c r="Y316" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z316" t="n">
+        <v>9985965602</v>
+      </c>
+      <c r="AA316" t="inlineStr"/>
+      <c r="AB316" t="inlineStr"/>
+      <c r="AC316" t="inlineStr"/>
+      <c r="AD316" t="inlineStr"/>
+      <c r="AE316" t="inlineStr"/>
+      <c r="AF316" t="inlineStr"/>
+      <c r="AG316" t="inlineStr"/>
+      <c r="AH316" t="inlineStr"/>
+      <c r="AI316" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ316" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK316" t="inlineStr"/>
+      <c r="AL316" t="inlineStr"/>
+      <c r="AM316" t="inlineStr"/>
+      <c r="AN316" t="inlineStr"/>
+      <c r="AO316" t="inlineStr"/>
+      <c r="AP316" t="inlineStr"/>
+      <c r="AQ316" t="inlineStr"/>
+      <c r="AR316" t="inlineStr"/>
+      <c r="AS316" t="inlineStr"/>
+      <c r="AT316" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU316" t="inlineStr"/>
+      <c r="AV316" t="inlineStr"/>
+      <c r="AW316" t="inlineStr"/>
+      <c r="AX316" t="inlineStr"/>
+      <c r="AY316" t="inlineStr"/>
+      <c r="AZ316" t="inlineStr"/>
+      <c r="BA316" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB316" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC316" t="inlineStr"/>
+      <c r="BD316" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE316" t="n">
+        <v>19941</v>
+      </c>
+      <c r="BF316" t="inlineStr">
+        <is>
+          <t>267541</t>
+        </is>
+      </c>
+      <c r="BG316" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="BH316" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI316" t="n">
+        <v>17229</v>
+      </c>
+      <c r="BJ316" t="inlineStr"/>
+      <c r="BK316" t="inlineStr"/>
+      <c r="BL316" t="inlineStr"/>
+      <c r="BM316" t="inlineStr"/>
+      <c r="BN316" t="inlineStr"/>
+      <c r="BO316" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+      <c r="BP316" t="inlineStr"/>
+      <c r="BQ316" t="inlineStr"/>
+      <c r="BR316" t="inlineStr"/>
+      <c r="BS316" t="inlineStr"/>
+      <c r="BT316" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU316" t="inlineStr"/>
+      <c r="BV316" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>753702</v>
+      </c>
+      <c r="C317" t="n">
+        <v>1234</v>
+      </c>
+      <c r="D317" t="n">
+        <v>11000349199255</v>
+      </c>
+      <c r="E317" t="n">
+        <v>1770541823</v>
+      </c>
+      <c r="F317" t="n">
+        <v>7750</v>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>08-Feb-2026 14:40:50</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N317" t="n">
+        <v>89695506546</v>
+      </c>
+      <c r="O317" t="inlineStr"/>
+      <c r="P317" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="Q317" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R317" t="inlineStr"/>
+      <c r="S317" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T317" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U317" t="inlineStr"/>
+      <c r="V317" t="inlineStr"/>
+      <c r="W317" t="inlineStr"/>
+      <c r="X317" t="inlineStr"/>
+      <c r="Y317" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z317" t="n">
+        <v>9866955786</v>
+      </c>
+      <c r="AA317" t="inlineStr"/>
+      <c r="AB317" t="inlineStr"/>
+      <c r="AC317" t="inlineStr"/>
+      <c r="AD317" t="inlineStr"/>
+      <c r="AE317" t="inlineStr"/>
+      <c r="AF317" t="inlineStr"/>
+      <c r="AG317" t="inlineStr"/>
+      <c r="AH317" t="inlineStr"/>
+      <c r="AI317" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ317" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK317" t="inlineStr"/>
+      <c r="AL317" t="inlineStr"/>
+      <c r="AM317" t="inlineStr"/>
+      <c r="AN317" t="inlineStr"/>
+      <c r="AO317" t="inlineStr"/>
+      <c r="AP317" t="inlineStr"/>
+      <c r="AQ317" t="inlineStr"/>
+      <c r="AR317" t="inlineStr"/>
+      <c r="AS317" t="inlineStr"/>
+      <c r="AT317" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU317" t="inlineStr"/>
+      <c r="AV317" t="inlineStr"/>
+      <c r="AW317" t="inlineStr"/>
+      <c r="AX317" t="inlineStr"/>
+      <c r="AY317" t="inlineStr"/>
+      <c r="AZ317" t="inlineStr"/>
+      <c r="BA317" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB317" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC317" t="inlineStr"/>
+      <c r="BD317" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE317" t="n">
+        <v>18265</v>
+      </c>
+      <c r="BF317" t="inlineStr">
+        <is>
+          <t>267000</t>
+        </is>
+      </c>
+      <c r="BG317" t="inlineStr">
+        <is>
+          <t>2056</t>
+        </is>
+      </c>
+      <c r="BH317" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI317" t="n">
+        <v>16342</v>
+      </c>
+      <c r="BJ317" t="inlineStr"/>
+      <c r="BK317" t="inlineStr"/>
+      <c r="BL317" t="inlineStr"/>
+      <c r="BM317" t="inlineStr"/>
+      <c r="BN317" t="inlineStr"/>
+      <c r="BO317" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+      <c r="BP317" t="inlineStr"/>
+      <c r="BQ317" t="inlineStr"/>
+      <c r="BR317" t="inlineStr"/>
+      <c r="BS317" t="inlineStr"/>
+      <c r="BT317" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU317" t="inlineStr"/>
+      <c r="BV317" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>